<commit_message>
enhnaced chatbot api. added list of answer, page num, source link
</commit_message>
<xml_diff>
--- a/src/s3/client_documents/circor_2_att6.xlsx
+++ b/src/s3/client_documents/circor_2_att6.xlsx
@@ -488,9 +488,9 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[3.1]: PT/MT &amp; Thickness verification for overlay &amp; hard facing. | 100% | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Inspection Report / NDT Reports, RT Films | H | W*/R | R | R | Review of RT films, RT, UT, PT reports to be provided for review for 100%. *10% witness by TPIA.
----
-[1.1]: Item No 1.1: Activity: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrottest, Pneumatic test, Heat Treatment procedures etc. (As applicable) | Extent of supply: 100% | Reference Document: API 598 ASME B 16.34 ASME Section V | Acceptance Criteria: API 598 ASME B 16.34 ASME Section V | Verifying Document: Approved NDT Procedures | Inspection Agency: Vendor H, TPIA R, LTEH R, OWNER/PMC R | Remarks: Duly approved by NDT level III person.</t>
+          <t>[3.1]: PT/MT &amp; Thickness verification for overlay &amp; hard facing.
+---
+[1.1]: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrot est, Pneumatic test, Heat Treatment procedures etc. (As applicable)|100%|API 598 ASME B 16.34 ASME Section V|API 598 ASME B 16.34 ASME Section V|Approved NDT Procedures|H|R|R|R|Duly approved by NDT level III person.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -524,7 +524,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[2.1]: 2.1|a) Material Identification and review of MTC for - 3.1 Mill test certificates as per EN 10204 for Valve Body, Bonnet, Plug, Seat, closure member &amp; trim material (Spray Head, Nozzle &amp; Spindle), Bar/ Forging &amp; Fasteners. 2.2 test certificate as per EN 10204 for non-pressure containing parts. b) IGC Test for all SS Material (As per approved datasheet)|100%|Approved MR, Datasheet, GAD's and applicable Specs ASTM/ASME/Standards.|Approved MR, Datasheet, GAD's and applicable Specs ASTM/ASME/Standards.|MTC's / Lab report / Heat Treatment Charts|H|R|R|R|</t>
+          <t>[2.1]: 2.1|a) Material Identification and review of MTC for - 3.1 Mill test certificates as per EN 10204 for Valve Body, Bonnet, Plug, Seat, closure member &amp; trim material (Spray Head, Nozzle &amp; Spindle), Bar/ Forging &amp; Fasteners. 2.2 test certificate as per EN 10204 for non-pressure containing parts. b) IGC Test for all SS Material (As per approved datasheet)|Approved MR, Datasheet, GAD's and applicable Specs ASTM/ASME/Standards.|Approved MR, Datasheet, GAD's and applicable Specs ASTM/ASME/Standards.|MTC's / Lab report / Heat Treatment Charts|H|R|R|R</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -541,7 +541,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[1.1]: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrottest, Pneumatic test, Heat Treatment procedures etc. (As applicable) | 100% | API 598 ASME B 16.34 ASME Section V | API 598 ASME B 16.34 ASME Section V | Approved NDT Procedures | H | R | R | R | Duly approved by NDT level III person.</t>
+          <t>[1.1]: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrot est, Pneumatic test, Heat Treatment procedures etc. (As applicable)|100%|API 598 ASME B 16.34 ASME Section V|API 598 ASME B 16.34 ASME Section V|Approved NDT Procedures|H|R|R|R|Duly approved by NDT level III person.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -575,11 +575,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[5.1]: Hydrostatic Shell Test: -At 1.5 times of max. Operating pressure. | Approved MR, Datasheet, GAD's and applicable Specs/ Standards. API-598 | Approved MR, Datasheet, GAD's and applicable Specs/ Standards. API-598 | Hydro test reports | P | RW | RW | R
----
-[5.2]: Hydrostatic Seat leakage test|100%|Approved MR, Datasheet, GAD's and applicable Specs/ Standards. API-598|Approved MR, Datasheet, GAD's and applicable Specs/ Standards. API-598|Hydro test reports|P|RW|RW|R
----
-[1.1]: Item No 1.1: Activity: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrotest, Pneumatic test, Heat Treatment procedures etc. (As applicable) | Reference Document: API 598 ASME B 16.34 ASME Section V | Acceptance Criteria: API 598 ASME B 16.34 ASME Section V | Verifying Document: Approved NDT Procedures</t>
+          <t>[5.1]: Hydrostatic Shell Test: -At 1.5 times of max. Operating pressure. | Approved MR, Datasheet, GAD's and applicable Specs/Standards. API-598 | Hydro test reports | P | RW | RW | R
+---
+[5.2]: Hydrostatic Seat leakage test | 100% | Approved MR, Datasheet, GAD's and applicable Specs/ Standards. API-598 | Approved MR, Datasheet, GAD's and applicable Specs/ Standards. API-598 | Hydro test reports | P | RW | RW | R
+---
+[1.1]: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrotest, Pneumatic test, Heat Treatment procedures etc. (As applicable) | API 598 | ASME B 16.34 | ASME Section V | Approved NDT Procedures | H | R | R | R | Duly approved by NDT level III person.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -596,9 +596,9 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>[2.1]: b) IGC Test for all SS Material (As per approved datasheet)
----
-[11]: For AS &amp; SS Material IGC test as per ASTM Practice "E" to be carried out, Additionally, Microscopic structure to be observed at 250X magnification for checking no carbide precipitation.</t>
+          <t>[2.1]: a) Material Identification and review of MTC for - 3.1 Mill test certificates as per EN 10204 for Valve Body, Bonnet, Plug, Seat, closure member &amp; trim material (Spray Head, Nozzle &amp; Spindle), Bar/ Forging &amp; Fasteners. 2.2 test certificate as per EN 10204 for non-pressure containing parts. b) IGC Test for all SS Material (As per approved datasheet)
+---
+[Note-6]: For AS &amp; SS Material IGC test as per ASTM Practice "E" to be carried out. Additionally, Microscopic structure to be observed at 250X magnification for checking no carbide precipitation.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -632,9 +632,9 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[3.3]: LPT/PT of Fillet weld Joint (As applicable)-soundness|100%|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Inspection Report / NDT Reports, RT Films|H|W*/R|R|R|Review of RT films, RT, UT, PT reports to be provided for review for 100%. *10% witness by TPIA.
----
-[1.1]: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrottest, Pneumatic test, Heat Treatment procedures etc. (As applicable)|API 598 ASME B 16.34 ASME Section V|API 598 ASME B 16.34 ASME Section V|Approved NDT Procedures|H|R|R|R|Duly approved by NDT level III person.</t>
+          <t>[3.3]: LPT/PT of Fillet weld Joint (As applicable)-soundness|100%|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Inspection Report / NDT Reports, RT Films|W*/R|R|R|Review of RT films, RT, UT, PT reports to be provided for review for 100%. *10% witness by TPIA.
+---
+[1.1]: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrot est, Pneumatic test, Heat Treatment procedures etc. (As applicable)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -651,14 +651,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[7.1]: 7.1|1. Manufacturer's test certificates for all bought out items, accessories &amp; spares etc. 2. Material co-relation chart showing Make, Model number, Sr Number, MTC/TC Number, Heat number, Statutory Certificate (As Applicable). Calibration &amp; Performance Certificates, NDT, Hydrottest, IBR certificates. other TCs &amp; Certificates as required by Data Sheets and Proj. Specs.|100%|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|MTC, TC's / reports|P|R|R|R|
----
-[1.1]: Item No 1.1 | Activity: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrot est, Pneumatic test, Heat Treatment procedures etc. (As applicable) | Extent of supply: 100% | Reference Document: API 598 ASME B 16.34 ASME Section V | Acceptance Criteria: API 598 ASME B 16.34 ASME Section V | Verifying Document: Approved NDT Procedures | Inspection Agency: Vendor H, TPIA R, LTEH R, OWNER/PMC R | Remarks: Duly approved by NDT level III person.</t>
+          <t>[1.1]: Item No 1.1: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrot est, Pneumatic test, Heat Treatment procedures etc. (As applicable) | Extent of supply: 100% | Reference Document: API 598 ASME B 16.34 ASME Section V | Acceptance Criteria: API 598 ASME B 16.34 ASME Section V | Verifying Document: Approved NDT Procedures | Inspection Agency: Vendor H, TPIA R, LTEH R, OWNER/PMC R | Remarks: Duly approved by NDT level III person.
+---
+[3.4]: UT for Forging, Bar stock (Trim Parts-Plug, Seat &amp; Spindle etc.) [above Ø50 mm]|100%|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Inspection Report / NDT Reports, RT Films|H|W*/R|R|R|Review of RT films, RT, UT, PT reports to be provided for review for 100%. *10% witness by TPIA.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5, 8</t>
+          <t>5, 6</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>[4]: PMI Test - All types of valves, rupture disks, bodies, pipe, flanges &amp; trim (Applicable for SS &amp; AS material), bonnets &amp; covers (as applicable)|100%|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|PMI reports|P|W*|R|R|100% PMI - review *10% PMI Witness</t>
+          <t>[4 PMI Test]: 4|PMI Test - All types of valves, rupture disks, bodies, pipe, flanges &amp; trim (Applicable for SS &amp; AS material), bonnets &amp; covers (as applicable)|100%|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|PMI reports|P|W*|R|R|100% PMI - review *10% PMI Witness</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -687,9 +687,9 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>[3.2]: RT of Butt weld Joint (As applicable) - soundness | 100% | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Inspection Report / NDT Reports, RT Films | H | W*/R | R | R | Review of RT films, RT, UT, PT reports to be provided for review for 100%. *10% witness by TPIA.
----
-[1.1]: Item No 1.1 | Activity: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrot est, Pneumatic test, Heat Treatment procedures etc. (As applicable) | Extent of supply: 100% | Reference Document: API 598 ASME B 16.34 ASME Section V | Acceptance Criteria: API 598 ASME B 16.34 ASME Section V | Verifying Document: Approved NDT Procedures | Inspection Agency: Vendor H, TPIA R, LTEH R, OWNER/PMC R | Remarks: Duly approved by NDT level III person.</t>
+          <t>[3.2]: RT of Butt weld Joint (As applicable) - soundness|100%|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Inspection Report / NDT Reports, RT Films|H|W*/R|R|R|Review of RT films, RT, UT, PT reports to be provided for review for 100%. *10% witness by TPIA.
+---
+[1.1]: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrot est, Pneumatic test, Heat Treatment procedures etc. (As applicable)|100%|API 598 ASME B 16.34 ASME Section V|API 598 ASME B 16.34 ASME Section V|Approved NDT Procedures|H|R|R|R|Duly approved by NDT level III person.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -706,9 +706,9 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>[3.4]: UT for Forging, Bar stock (Trim Parts-Plug, Seat &amp; Spindle etc.) (above Ø50 mm)|100%|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Inspection Report / NDT Reports, RT Films|H|W*/R|R|R|Review of RT films, RT, UT, PT reports to be provided for review for 100%. *10% witness by TPIA.
----
-[1.1]: Item No 1.1 | Activity: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrottest, Pneumatic test, Heat Treatment procedures etc. (As applicable) | Extent of supply: 100% | Reference Document: API 598 ASME B 16.34 ASME Section V | Acceptance Criteria: API 598 ASME B 16.34 ASME Section V | Verifying Document: Approved NDT Procedures | Inspection Agency: Vendor H, TPIA R, LTEH R, OWNER/PMC R | Remarks: Duly approved by NDT level III person.</t>
+          <t>[3.4]: UT for Forging, Bar stock (Trim Parts-Plug, Seat &amp; Spindle etc.) [above Ø50 mm]|100%|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Approved MR, Datasheet, GAD's and applicable Specs/Standards.|Inspection Report / NDT Reports, RT Films|H|W*/R|R|R|Review of RT films, RT, UT, PT reports to be provided for review for 100%. *10% witness by TPIA.
+---
+[1.1]: NDT / QA-QC Procedures: DPT, MT, RT, UT Hydrot est, Pneumatic test, Heat Treatment procedures etc. (As applicable)|100%|API 598 ASME B 16.34 ASME Section V|API 598 ASME B 16.34 ASME Section V|Approved NDT Procedures|H|R|R|R|Duly approved by NDT level III person.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[1.2]: WPS / PQR / WPQ for welded valves, Overlay, Stellite &amp; Weld repair (As applicable) | 100% | ASME Section IX | ASME Section IX | Approved WPS, PQR &amp; WPQ | H | R | R | R | Duly certified by Reputed TPIA</t>
+          <t>[1.2]: WPS / PQR / WPQ for welded valves, Overlay, Stellite &amp; Weld repair (As applicable)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -759,13 +759,13 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>[3 Definitions]: Perform Point "P"|Manufacturer / Supplier shall 100% perform inspection check.|Hold Point "H"|Hold for Inspection and do not proceed. Fabrication shall be kept under hold until inspection has been performed or written clearance is obtained by Vendor. The work cannot proceed unless the Hold Point is cleared.|Witness Point "W"|Witness for Inspection Advise of inspection, Fabrication may be continued if inspector is not present after invitation issued in due time.|Review Point "R"|Review / Check / Verify documents. Review of Procedures / Test Reports / Certificates / Inspection Reports
----
-[5.7]: Performance Check: Functional test of complete assembly (as applicable). Functional/Calibration Test on Valve, Positioner/Robotor, Actuator &amp; Hand wheel &amp; accessories mounted. (Stroke, Linearity &amp; Hysteresis) Paint shade &amp; DFT check | 100% | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Inspection reports | P | W | W | R
----
-[3.5]: Physical &amp; Visual Checks which includes: Markings, Overall dimensions, Face to face body dimension, Flanges verification, Thickness check, Checks for accessories, connections &amp; installations. Functional checks on complete valve with all accessories. | 100% | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Inspection Report | H | W | R | R | Review of RT films, RT, UT, PT reports to be provided for review for 100%. *10% witness by TPIA.
----
-[7.1]: Item No 7.1: Documents Review. Activity: 1. Manufacturer's test certificates for all bought out items, accessories &amp; spares etc. 2. Material co-relation chart showing Make, Model number, Sr Number, MTC/TC Number, Heat number, Statutory Certificate (As Applicable). Calibration &amp; Performance Certificates, NDT, Hydrotect, IBR certificates. other TCs &amp; Certificates as required by Data Sheets and Proj. Specs. Extent of supply: 100%. Reference Document: Approved MR, Datasheet, GAD's and applicable Specs/Standards. Acceptance Criteria: Approved MR, Datasheet, GAD's and applicable Specs/Standards. Verifying Document: MTC, TC's / reports. Inspection Agency: Vendor-P, TPIA-R, LTEH-R, OWNER/PMC-R. Remarks: None.</t>
+          <t>[3 Definitions]: Perform Point "P" | Manufacturer / Supplier shall 100% perform inspection check. Hold Point "H" | Hold for Inspection and do not proceed. Fabrication shall be kept under hold until inspection has been performed or written clearance is obtained by Vendor. The work cannot proceed unless the Hold Point is cleared. Witness Point "W" | Witness for Inspection | Advise of inspection, Fabrication may be continued if inspector is not present after invitation issued in due time. Review Point "R" | Review / Check / Verify documents. | Review of Procedures / Test Reports / Certificates / Inspection Reports
+---
+[3]: In Process Inspection- | PT/MT &amp; Thickness verification for overlay &amp; hard facing. | 100% | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Inspection Report / NDT Reports, RT Films | H | W*/R | R | R | Review of RT films, RT, UT, PT reports to be provided for review for 100%. *10% witness by TPIA. | RT of Butt weld Joint (As applicable) - soundness | 100% | LPT/PT of Fillet weld Joint (As applicable)-soundness | 100% | UT for Forging, Bar stock (Trim Parts- Plug, Seat &amp; Spindle etc.) [above Ø50 mm] | 100% | Physical &amp; Visual Checks which includes: Markings, Overall dimensions, Face to face body dimension, Flanges verification, Thickness check, Checks for accessories, connections &amp; installations. Functional checks on complete valve with all accessories. | 100% | Inspection Report | H | W | R | R
+---
+[5.7]: Performance Check: Functional test of complete assembly (as applicable). Functional/Calibration Test on Valve, Positioner/Robotor, Actuator &amp; Hand wheel &amp; accessories mounted. (Stroke, Linearity &amp; Hysteresis) Paint shade &amp; DFT check | 100% | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Inspection reports | W | W | R
+---
+[7 Documents Review]: 7.1. Manufacturer's test certificates for all bought out items, accessories &amp; spares etc. | 100% | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | Approved MR, Datasheet, GAD's and applicable Specs/Standards. | MTC, TC's / reports | P | R | R | R</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -782,15 +782,15 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>[]: No relevant information found
+          <t>[No relevant information found]: No relevant information found
 ---
 []: No relevant information found
 ---
+[No relevant information found]: No relevant information found
+---
 []: No relevant information found
 ---
-[2.1]: Material Identification and review of MTC for - 3.1 Mill test certificates as per EN 10204 for Valve Body, Bonnet, Plug, Seat, closure member &amp; trim material (Spray Head, Nozzle &amp; Spindle), Bar/ Forging &amp; Fasteners. 2.2 test certificate as per EN 10204 for non-pressure containing parts. b) IGC Test for all SS Material (As per approved datasheet) | 100% | Approved MR, Datasheet, GAD's and applicable Specs ASTM/ASME/Standards. | Approved MR, Datasheet, GAD's and applicable Specs ASTM/ASME/Standards. | MTC's / Lab report / Heat Treatment Charts | H | R | R | R
----
-[]: No relevant information found</t>
+[2.1]: Material Identification and review of MTC for - 3.1 Mill test certificates as per EN 10204 for Valve Body, Bonnet, Plug, Seat, closure member &amp; trim material (Spray Head, Nozzle &amp; Spindle), Bar/ Forging &amp; Fasteners. 2.2 test certificate as per EN 10204 for non-pressure containing parts. b) IGC Test for all SS Material (As per approved datasheet)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">

</xml_diff>